<commit_message>
add auto phase change
</commit_message>
<xml_diff>
--- a/RL/job_logs.xlsx
+++ b/RL/job_logs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,20 +513,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-11-04 01:20:45</t>
+          <t>2025-12-22 18:54:32</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>0.0001</v>
       </c>
       <c r="D2" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="E2" t="n">
-        <v>256</v>
+        <v>64</v>
       </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G2" t="n">
         <v>0.99</v>
@@ -541,10 +541,10 @@
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>20000</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -570,20 +570,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-11-04 16:23:46</t>
+          <t>2025-12-22 20:41:07</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>0.0001</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>1024</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
         <v>0.99</v>
@@ -598,10 +598,10 @@
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L3" t="n">
-        <v>100</v>
+        <v>9000</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -614,234 +614,6 @@
         </is>
       </c>
       <c r="O3" t="inlineStr">
-        <is>
-          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>jobid</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-11-04 16:46:35</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="n">
-        <v>85</v>
-      </c>
-      <c r="L4" t="n">
-        <v>100</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>model_jobid</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>./tensorboard/model_jobid</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>jobid</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2025-11-04 16:49:23</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>15</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>85</v>
-      </c>
-      <c r="L5" t="n">
-        <v>200</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>model_jobid</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>./tensorboard/model_jobid</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>jobid</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2025-11-04 16:54:16</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="n">
-        <v>85</v>
-      </c>
-      <c r="L6" t="n">
-        <v>200</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>model_jobid</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>./tensorboard/model_jobid</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>jobid</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2025-11-04 16:57:47</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="n">
-        <v>15</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" t="n">
-        <v>85</v>
-      </c>
-      <c r="L7" t="n">
-        <v>200</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>model_jobid</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>./tensorboard/model_jobid</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
         <is>
           <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
         </is>

</xml_diff>

<commit_message>
fix the rotation guard issue
</commit_message>
<xml_diff>
--- a/RL/job_logs.xlsx
+++ b/RL/job_logs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -904,6 +904,405 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-14 12:10:21</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E9" t="n">
+        <v>128</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-14 12:12:14</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E10" t="n">
+        <v>128</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-14 12:22:41</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E11" t="n">
+        <v>128</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-04-15 22:05:02</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E12" t="n">
+        <v>128</v>
+      </c>
+      <c r="F12" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-15 22:14:47</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E13" t="n">
+        <v>128</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>8</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-15 22:16:59</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E14" t="n">
+        <v>128</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>8</v>
+      </c>
+      <c r="L14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-15 22:18:50</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E15" t="n">
+        <v>128</v>
+      </c>
+      <c r="F15" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>model_jobid</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>